<commit_message>
Correction des profiles suite aux erreurs qa dans IPS FR 076636519a3fbcf93c7296f17f51d80164ae8a4f
</commit_message>
<xml_diff>
--- a/correctionProfile/ig/StructureDefinition-fr-composition-document.xlsx
+++ b/correctionProfile/ig/StructureDefinition-fr-composition-document.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9890" uniqueCount="907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9890" uniqueCount="908">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-17T15:33:46+00:00</t>
+    <t>2026-09-28T13:37:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2474,6 +2474,10 @@
     <t>Provides context for the composition and creates a linkage between a resource describing an event and the composition created describing the event.</t>
   </si>
   <si>
+    <t xml:space="preserve">exists:$this}
+</t>
+  </si>
+  <si>
     <t>outboundRelationship[typeCode="SUBJ"].target[classCode&lt;'ACT']</t>
   </si>
   <si>
@@ -2603,7 +2607,7 @@
   </si>
   <si>
     <t>cmp-1:A section must contain at least one of text, entries, or sub-sections {text.exists() or entry.exists() or section.exists()}
-cmp-2:A section can only have an emptyReason if it is empty {emptyReason.empty() or entry.empty()}ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}comp-4:Une section ne peut pas contenir à la fois des entrées et des sous-sections. {not(exists(f:entry) and exists(f:section))}</t>
+cmp-2:A section can only have an emptyReason if it is empty {emptyReason.empty() or entry.empty()}ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}comp-4:Une section ne peut pas contenir à la fois des entrées et des sous-sections. {entry.exists().not() or section.exists().not()}</t>
   </si>
   <si>
     <t>./outboundRelationship[typeCode="COMP" and isNormalActRelationship()]/target[moodCode="EVN" and classCode="DOCSECT" and isNormalAct]</t>
@@ -30770,7 +30774,7 @@
         <v>78</v>
       </c>
       <c r="AB237" t="s" s="2">
-        <v>143</v>
+        <v>788</v>
       </c>
       <c r="AC237" s="2"/>
       <c r="AD237" t="s" s="2">
@@ -30798,13 +30802,13 @@
         <v>78</v>
       </c>
       <c r="AL237" t="s" s="2">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="AM237" t="s" s="2">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="AN237" t="s" s="2">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="AO237" t="s" s="2">
         <v>78</v>
@@ -30812,10 +30816,10 @@
     </row>
     <row r="238" hidden="true">
       <c r="A238" t="s" s="2">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B238" t="s" s="2">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="C238" s="2"/>
       <c r="D238" t="s" s="2">
@@ -30927,10 +30931,10 @@
     </row>
     <row r="239" hidden="true">
       <c r="A239" t="s" s="2">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="B239" t="s" s="2">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="C239" s="2"/>
       <c r="D239" t="s" s="2">
@@ -31040,13 +31044,13 @@
     </row>
     <row r="240" hidden="true">
       <c r="A240" t="s" s="2">
+        <v>794</v>
+      </c>
+      <c r="B240" t="s" s="2">
         <v>793</v>
       </c>
-      <c r="B240" t="s" s="2">
-        <v>792</v>
-      </c>
       <c r="C240" t="s" s="2">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="D240" t="s" s="2">
         <v>78</v>
@@ -31068,13 +31072,13 @@
         <v>78</v>
       </c>
       <c r="K240" t="s" s="2">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="L240" t="s" s="2">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="M240" t="s" s="2">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="N240" s="2"/>
       <c r="O240" s="2"/>
@@ -31157,10 +31161,10 @@
     </row>
     <row r="241" hidden="true">
       <c r="A241" t="s" s="2">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="C241" s="2"/>
       <c r="D241" t="s" s="2">
@@ -31276,10 +31280,10 @@
     </row>
     <row r="242" hidden="true">
       <c r="A242" t="s" s="2">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="C242" s="2"/>
       <c r="D242" t="s" s="2">
@@ -31305,13 +31309,13 @@
         <v>237</v>
       </c>
       <c r="L242" t="s" s="2">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="M242" t="s" s="2">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="N242" t="s" s="2">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="O242" s="2"/>
       <c r="P242" t="s" s="2">
@@ -31340,10 +31344,10 @@
         <v>163</v>
       </c>
       <c r="Y242" t="s" s="2">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="Z242" t="s" s="2">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="AA242" t="s" s="2">
         <v>78</v>
@@ -31361,7 +31365,7 @@
         <v>78</v>
       </c>
       <c r="AF242" t="s" s="2">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="AG242" t="s" s="2">
         <v>79</v>
@@ -31385,7 +31389,7 @@
         <v>472</v>
       </c>
       <c r="AN242" t="s" s="2">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="AO242" t="s" s="2">
         <v>78</v>
@@ -31393,10 +31397,10 @@
     </row>
     <row r="243" hidden="true">
       <c r="A243" t="s" s="2">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="B243" t="s" s="2">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="C243" s="2"/>
       <c r="D243" t="s" s="2">
@@ -31422,10 +31426,10 @@
         <v>261</v>
       </c>
       <c r="L243" t="s" s="2">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="M243" t="s" s="2">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="N243" s="2"/>
       <c r="O243" s="2"/>
@@ -31476,7 +31480,7 @@
         <v>78</v>
       </c>
       <c r="AF243" t="s" s="2">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="AG243" t="s" s="2">
         <v>79</v>
@@ -31500,7 +31504,7 @@
         <v>543</v>
       </c>
       <c r="AN243" t="s" s="2">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="AO243" t="s" s="2">
         <v>78</v>
@@ -31508,10 +31512,10 @@
     </row>
     <row r="244" hidden="true">
       <c r="A244" t="s" s="2">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="B244" t="s" s="2">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="C244" s="2"/>
       <c r="D244" t="s" s="2">
@@ -31534,13 +31538,13 @@
         <v>92</v>
       </c>
       <c r="K244" t="s" s="2">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="L244" t="s" s="2">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="M244" t="s" s="2">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="N244" s="2"/>
       <c r="O244" s="2"/>
@@ -31591,7 +31595,7 @@
         <v>78</v>
       </c>
       <c r="AF244" t="s" s="2">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="AG244" t="s" s="2">
         <v>79</v>
@@ -31609,7 +31613,7 @@
         <v>78</v>
       </c>
       <c r="AL244" t="s" s="2">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="AM244" t="s" s="2">
         <v>109</v>
@@ -31623,13 +31627,13 @@
     </row>
     <row r="245" hidden="true">
       <c r="A245" t="s" s="2">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B245" t="s" s="2">
         <v>783</v>
       </c>
       <c r="C245" t="s" s="2">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="D245" t="s" s="2">
         <v>78</v>
@@ -31654,7 +31658,7 @@
         <v>582</v>
       </c>
       <c r="L245" t="s" s="2">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="M245" t="s" s="2">
         <v>785</v>
@@ -31730,13 +31734,13 @@
         <v>78</v>
       </c>
       <c r="AL245" t="s" s="2">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="AM245" t="s" s="2">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="AN245" t="s" s="2">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="AO245" t="s" s="2">
         <v>78</v>
@@ -31744,10 +31748,10 @@
     </row>
     <row r="246" hidden="true">
       <c r="A246" t="s" s="2">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="B246" t="s" s="2">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="C246" s="2"/>
       <c r="D246" t="s" s="2">
@@ -31859,10 +31863,10 @@
     </row>
     <row r="247" hidden="true">
       <c r="A247" t="s" s="2">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="B247" t="s" s="2">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="C247" s="2"/>
       <c r="D247" t="s" s="2">
@@ -31972,13 +31976,13 @@
     </row>
     <row r="248" hidden="true">
       <c r="A248" t="s" s="2">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="B248" t="s" s="2">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="C248" t="s" s="2">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="D248" t="s" s="2">
         <v>78</v>
@@ -32000,13 +32004,13 @@
         <v>78</v>
       </c>
       <c r="K248" t="s" s="2">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="L248" t="s" s="2">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="M248" t="s" s="2">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="N248" s="2"/>
       <c r="O248" s="2"/>
@@ -32089,10 +32093,10 @@
     </row>
     <row r="249" hidden="true">
       <c r="A249" t="s" s="2">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B249" t="s" s="2">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="C249" s="2"/>
       <c r="D249" t="s" s="2">
@@ -32208,10 +32212,10 @@
     </row>
     <row r="250" hidden="true">
       <c r="A250" t="s" s="2">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="B250" t="s" s="2">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="C250" s="2"/>
       <c r="D250" t="s" s="2">
@@ -32237,13 +32241,13 @@
         <v>237</v>
       </c>
       <c r="L250" t="s" s="2">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="M250" t="s" s="2">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="N250" t="s" s="2">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="O250" s="2"/>
       <c r="P250" t="s" s="2">
@@ -32272,10 +32276,10 @@
         <v>163</v>
       </c>
       <c r="Y250" t="s" s="2">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="Z250" t="s" s="2">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="AA250" t="s" s="2">
         <v>78</v>
@@ -32293,7 +32297,7 @@
         <v>78</v>
       </c>
       <c r="AF250" t="s" s="2">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="AG250" t="s" s="2">
         <v>79</v>
@@ -32317,7 +32321,7 @@
         <v>472</v>
       </c>
       <c r="AN250" t="s" s="2">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="AO250" t="s" s="2">
         <v>78</v>
@@ -32325,10 +32329,10 @@
     </row>
     <row r="251" hidden="true">
       <c r="A251" t="s" s="2">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="B251" t="s" s="2">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="C251" s="2"/>
       <c r="D251" t="s" s="2">
@@ -32354,10 +32358,10 @@
         <v>261</v>
       </c>
       <c r="L251" t="s" s="2">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="M251" t="s" s="2">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="N251" s="2"/>
       <c r="O251" s="2"/>
@@ -32408,7 +32412,7 @@
         <v>78</v>
       </c>
       <c r="AF251" t="s" s="2">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="AG251" t="s" s="2">
         <v>79</v>
@@ -32432,7 +32436,7 @@
         <v>543</v>
       </c>
       <c r="AN251" t="s" s="2">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="AO251" t="s" s="2">
         <v>78</v>
@@ -32440,10 +32444,10 @@
     </row>
     <row r="252" hidden="true">
       <c r="A252" t="s" s="2">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="B252" t="s" s="2">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="C252" s="2"/>
       <c r="D252" t="s" s="2">
@@ -32466,13 +32470,13 @@
         <v>92</v>
       </c>
       <c r="K252" t="s" s="2">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="L252" t="s" s="2">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="M252" t="s" s="2">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="N252" s="2"/>
       <c r="O252" s="2"/>
@@ -32523,7 +32527,7 @@
         <v>78</v>
       </c>
       <c r="AF252" t="s" s="2">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="AG252" t="s" s="2">
         <v>79</v>
@@ -32541,7 +32545,7 @@
         <v>78</v>
       </c>
       <c r="AL252" t="s" s="2">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="AM252" t="s" s="2">
         <v>109</v>
@@ -32555,10 +32559,10 @@
     </row>
     <row r="253">
       <c r="A253" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="B253" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="C253" s="2"/>
       <c r="D253" t="s" s="2">
@@ -32584,10 +32588,10 @@
         <v>582</v>
       </c>
       <c r="L253" t="s" s="2">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="M253" t="s" s="2">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="N253" s="2"/>
       <c r="O253" s="2"/>
@@ -32638,7 +32642,7 @@
         <v>78</v>
       </c>
       <c r="AF253" t="s" s="2">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="AG253" t="s" s="2">
         <v>79</v>
@@ -32650,16 +32654,16 @@
         <v>78</v>
       </c>
       <c r="AJ253" t="s" s="2">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="AK253" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL253" t="s" s="2">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="AM253" t="s" s="2">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="AN253" t="s" s="2">
         <v>78</v>
@@ -32670,10 +32674,10 @@
     </row>
     <row r="254" hidden="true">
       <c r="A254" t="s" s="2">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="B254" t="s" s="2">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="C254" s="2"/>
       <c r="D254" t="s" s="2">
@@ -32785,10 +32789,10 @@
     </row>
     <row r="255" hidden="true">
       <c r="A255" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B255" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C255" s="2"/>
       <c r="D255" t="s" s="2">
@@ -32898,10 +32902,10 @@
     </row>
     <row r="256" hidden="true">
       <c r="A256" t="s" s="2">
+        <v>836</v>
+      </c>
+      <c r="B256" t="s" s="2">
         <v>835</v>
-      </c>
-      <c r="B256" t="s" s="2">
-        <v>834</v>
       </c>
       <c r="C256" t="s" s="2">
         <v>407</v>
@@ -32929,7 +32933,7 @@
         <v>409</v>
       </c>
       <c r="L256" t="s" s="2">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="M256" t="s" s="2">
         <v>410</v>
@@ -33015,13 +33019,13 @@
     </row>
     <row r="257" hidden="true">
       <c r="A257" t="s" s="2">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="B257" t="s" s="2">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="C257" t="s" s="2">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="D257" t="s" s="2">
         <v>78</v>
@@ -33043,16 +33047,16 @@
         <v>78</v>
       </c>
       <c r="K257" t="s" s="2">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="L257" t="s" s="2">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="M257" t="s" s="2">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="N257" t="s" s="2">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="O257" s="2"/>
       <c r="P257" t="s" s="2">
@@ -33134,10 +33138,10 @@
     </row>
     <row r="258" hidden="true">
       <c r="A258" t="s" s="2">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="B258" t="s" s="2">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="C258" s="2"/>
       <c r="D258" t="s" s="2">
@@ -33253,14 +33257,14 @@
     </row>
     <row r="259">
       <c r="A259" t="s" s="2">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B259" t="s" s="2">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="C259" s="2"/>
       <c r="D259" t="s" s="2">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="E259" s="2"/>
       <c r="F259" t="s" s="2">
@@ -33282,16 +33286,16 @@
         <v>105</v>
       </c>
       <c r="L259" t="s" s="2">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="M259" t="s" s="2">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="N259" t="s" s="2">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="O259" t="s" s="2">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="P259" t="s" s="2">
         <v>78</v>
@@ -33340,7 +33344,7 @@
         <v>78</v>
       </c>
       <c r="AF259" t="s" s="2">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="AG259" t="s" s="2">
         <v>79</v>
@@ -33372,10 +33376,10 @@
     </row>
     <row r="260">
       <c r="A260" t="s" s="2">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="B260" t="s" s="2">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="C260" s="2"/>
       <c r="D260" t="s" s="2">
@@ -33401,16 +33405,16 @@
         <v>237</v>
       </c>
       <c r="L260" t="s" s="2">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="M260" t="s" s="2">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="N260" t="s" s="2">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="O260" t="s" s="2">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="P260" t="s" s="2">
         <v>78</v>
@@ -33439,7 +33443,7 @@
       </c>
       <c r="Y260" s="2"/>
       <c r="Z260" t="s" s="2">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="AA260" t="s" s="2">
         <v>78</v>
@@ -33457,7 +33461,7 @@
         <v>78</v>
       </c>
       <c r="AF260" t="s" s="2">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="AG260" t="s" s="2">
         <v>79</v>
@@ -33489,10 +33493,10 @@
     </row>
     <row r="261" hidden="true">
       <c r="A261" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B261" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="C261" s="2"/>
       <c r="D261" t="s" s="2">
@@ -33515,13 +33519,13 @@
         <v>78</v>
       </c>
       <c r="K261" t="s" s="2">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="L261" t="s" s="2">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="M261" t="s" s="2">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="N261" s="2"/>
       <c r="O261" t="s" s="2">
@@ -33574,7 +33578,7 @@
         <v>78</v>
       </c>
       <c r="AF261" t="s" s="2">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="AG261" t="s" s="2">
         <v>79</v>
@@ -33606,10 +33610,10 @@
     </row>
     <row r="262" hidden="true">
       <c r="A262" t="s" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="B262" t="s" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C262" s="2"/>
       <c r="D262" t="s" s="2">
@@ -33632,16 +33636,16 @@
         <v>78</v>
       </c>
       <c r="K262" t="s" s="2">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="L262" t="s" s="2">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="M262" t="s" s="2">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="N262" t="s" s="2">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="O262" s="2"/>
       <c r="P262" t="s" s="2">
@@ -33691,7 +33695,7 @@
         <v>78</v>
       </c>
       <c r="AF262" t="s" s="2">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="AG262" t="s" s="2">
         <v>79</v>
@@ -33712,7 +33716,7 @@
         <v>78</v>
       </c>
       <c r="AM262" t="s" s="2">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="AN262" t="s" s="2">
         <v>78</v>
@@ -33723,10 +33727,10 @@
     </row>
     <row r="263">
       <c r="A263" t="s" s="2">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B263" t="s" s="2">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="C263" s="2"/>
       <c r="D263" t="s" s="2">
@@ -33752,13 +33756,13 @@
         <v>184</v>
       </c>
       <c r="L263" t="s" s="2">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="M263" t="s" s="2">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="N263" t="s" s="2">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="O263" s="2"/>
       <c r="P263" t="s" s="2">
@@ -33808,7 +33812,7 @@
         <v>78</v>
       </c>
       <c r="AF263" t="s" s="2">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="AG263" t="s" s="2">
         <v>79</v>
@@ -33817,7 +33821,7 @@
         <v>91</v>
       </c>
       <c r="AI263" t="s" s="2">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="AJ263" t="s" s="2">
         <v>103</v>
@@ -33826,10 +33830,10 @@
         <v>78</v>
       </c>
       <c r="AL263" t="s" s="2">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="AM263" t="s" s="2">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="AN263" t="s" s="2">
         <v>78</v>
@@ -33840,10 +33844,10 @@
     </row>
     <row r="264" hidden="true">
       <c r="A264" t="s" s="2">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B264" t="s" s="2">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="C264" s="2"/>
       <c r="D264" t="s" s="2">
@@ -33869,16 +33873,16 @@
         <v>173</v>
       </c>
       <c r="L264" t="s" s="2">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="M264" t="s" s="2">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="N264" t="s" s="2">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="O264" t="s" s="2">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="P264" t="s" s="2">
         <v>78</v>
@@ -33906,10 +33910,10 @@
         <v>327</v>
       </c>
       <c r="Y264" t="s" s="2">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="Z264" t="s" s="2">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="AA264" t="s" s="2">
         <v>78</v>
@@ -33927,7 +33931,7 @@
         <v>78</v>
       </c>
       <c r="AF264" t="s" s="2">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="AG264" t="s" s="2">
         <v>79</v>
@@ -33945,7 +33949,7 @@
         <v>78</v>
       </c>
       <c r="AL264" t="s" s="2">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="AM264" t="s" s="2">
         <v>109</v>
@@ -33959,10 +33963,10 @@
     </row>
     <row r="265" hidden="true">
       <c r="A265" t="s" s="2">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="B265" t="s" s="2">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="C265" s="2"/>
       <c r="D265" t="s" s="2">
@@ -33988,16 +33992,16 @@
         <v>237</v>
       </c>
       <c r="L265" t="s" s="2">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="M265" t="s" s="2">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="N265" t="s" s="2">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="O265" t="s" s="2">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="P265" t="s" s="2">
         <v>78</v>
@@ -34025,10 +34029,10 @@
         <v>177</v>
       </c>
       <c r="Y265" t="s" s="2">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="Z265" t="s" s="2">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="AA265" t="s" s="2">
         <v>78</v>
@@ -34046,7 +34050,7 @@
         <v>78</v>
       </c>
       <c r="AF265" t="s" s="2">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="AG265" t="s" s="2">
         <v>79</v>
@@ -34064,7 +34068,7 @@
         <v>78</v>
       </c>
       <c r="AL265" t="s" s="2">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="AM265" t="s" s="2">
         <v>109</v>
@@ -34078,10 +34082,10 @@
     </row>
     <row r="266" hidden="true">
       <c r="A266" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="B266" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C266" s="2"/>
       <c r="D266" t="s" s="2">
@@ -34104,16 +34108,16 @@
         <v>78</v>
       </c>
       <c r="K266" t="s" s="2">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="L266" t="s" s="2">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="M266" t="s" s="2">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="N266" t="s" s="2">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="O266" s="2"/>
       <c r="P266" t="s" s="2">
@@ -34163,7 +34167,7 @@
         <v>78</v>
       </c>
       <c r="AF266" t="s" s="2">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="AG266" t="s" s="2">
         <v>79</v>
@@ -34172,7 +34176,7 @@
         <v>80</v>
       </c>
       <c r="AI266" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="AJ266" t="s" s="2">
         <v>103</v>
@@ -34181,10 +34185,10 @@
         <v>78</v>
       </c>
       <c r="AL266" t="s" s="2">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="AM266" t="s" s="2">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="AN266" t="s" s="2">
         <v>78</v>
@@ -34195,10 +34199,10 @@
     </row>
     <row r="267" hidden="true">
       <c r="A267" t="s" s="2">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="B267" t="s" s="2">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="C267" s="2"/>
       <c r="D267" t="s" s="2">
@@ -34224,16 +34228,16 @@
         <v>237</v>
       </c>
       <c r="L267" t="s" s="2">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="M267" t="s" s="2">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="N267" t="s" s="2">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="O267" t="s" s="2">
-        <v>898</v>
+        <v>899</v>
       </c>
       <c r="P267" t="s" s="2">
         <v>78</v>
@@ -34261,10 +34265,10 @@
         <v>177</v>
       </c>
       <c r="Y267" t="s" s="2">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="Z267" t="s" s="2">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="AA267" t="s" s="2">
         <v>78</v>
@@ -34282,7 +34286,7 @@
         <v>78</v>
       </c>
       <c r="AF267" t="s" s="2">
-        <v>894</v>
+        <v>895</v>
       </c>
       <c r="AG267" t="s" s="2">
         <v>79</v>
@@ -34291,7 +34295,7 @@
         <v>91</v>
       </c>
       <c r="AI267" t="s" s="2">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="AJ267" t="s" s="2">
         <v>103</v>
@@ -34300,7 +34304,7 @@
         <v>78</v>
       </c>
       <c r="AL267" t="s" s="2">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="AM267" t="s" s="2">
         <v>109</v>
@@ -34314,10 +34318,10 @@
     </row>
     <row r="268" hidden="true">
       <c r="A268" t="s" s="2">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="B268" t="s" s="2">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="C268" s="2"/>
       <c r="D268" t="s" s="2">
@@ -34343,13 +34347,13 @@
         <v>81</v>
       </c>
       <c r="L268" t="s" s="2">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="M268" t="s" s="2">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="N268" t="s" s="2">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="O268" s="2"/>
       <c r="P268" t="s" s="2">
@@ -34399,7 +34403,7 @@
         <v>78</v>
       </c>
       <c r="AF268" t="s" s="2">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="AG268" t="s" s="2">
         <v>79</v>
@@ -34408,7 +34412,7 @@
         <v>80</v>
       </c>
       <c r="AI268" t="s" s="2">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="AJ268" t="s" s="2">
         <v>103</v>
@@ -34417,10 +34421,10 @@
         <v>78</v>
       </c>
       <c r="AL268" t="s" s="2">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="AM268" t="s" s="2">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="AN268" t="s" s="2">
         <v>78</v>

</xml_diff>

<commit_message>
Mise à jour des profils suites aux issues et retour NRISS 0f171b30bc0033a60f0c74806713ebaaa25dcfa7
</commit_message>
<xml_diff>
--- a/correctionProfile/ig/StructureDefinition-fr-composition-document.xlsx
+++ b/correctionProfile/ig/StructureDefinition-fr-composition-document.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$268</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AO$274</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9890" uniqueCount="908">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10109" uniqueCount="925">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-29T09:01:26+00:00</t>
+    <t>2026-09-30T14:16:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2474,7 +2474,7 @@
     <t>Provides context for the composition and creates a linkage between a resource describing an event and the composition created describing the event.</t>
   </si>
   <si>
-    <t xml:space="preserve">exists:$this}
+    <t xml:space="preserve">value:extension('https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-is-principal-event-extension').value}
 </t>
   </si>
   <si>
@@ -2509,6 +2509,22 @@
     <t>Extension permettant d'ajouter l'exécutant de l'évènement documenté. Ajout d'un performer à l'élément event d'une Composition.</t>
   </si>
   <si>
+    <t>Composition.event.extension:isPrincipal</t>
+  </si>
+  <si>
+    <t>isPrincipal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-is-principal-event-extension|0.1.0}
+</t>
+  </si>
+  <si>
+    <t>Indique si l'évènement documenté est l'évènement principal</t>
+  </si>
+  <si>
+    <t>Extension permettant d'indiquer si l'évènement documenté est l'évènement documenté principal. Vaut true pour l'évènement principal. Ajout d'un indicateur à l'élément event d'une Composition.</t>
+  </si>
+  <si>
     <t>Composition.event.modifierExtension</t>
   </si>
   <si>
@@ -2580,6 +2596,43 @@
   </si>
   <si>
     <t>Exécutant de l'évènement documenté principal</t>
+  </si>
+  <si>
+    <t>Composition.event:principalEvent.extension:isPrincipal</t>
+  </si>
+  <si>
+    <t>Composition.event:principalEvent.extension:isPrincipal.id</t>
+  </si>
+  <si>
+    <t>Composition.event.extension.id</t>
+  </si>
+  <si>
+    <t>Composition.event:principalEvent.extension:isPrincipal.extension</t>
+  </si>
+  <si>
+    <t>Composition.event.extension.extension</t>
+  </si>
+  <si>
+    <t>Composition.event:principalEvent.extension:isPrincipal.url</t>
+  </si>
+  <si>
+    <t>Composition.event.extension.url</t>
+  </si>
+  <si>
+    <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-is-principal-event-extension</t>
+  </si>
+  <si>
+    <t>Composition.event:principalEvent.extension:isPrincipal.value[x]</t>
+  </si>
+  <si>
+    <t>Composition.event.extension.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">boolean
+</t>
+  </si>
+  <si>
+    <t>true</t>
   </si>
   <si>
     <t>Composition.event:principalEvent.modifierExtension</t>
@@ -3158,7 +3211,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AO268"/>
+  <dimension ref="A1:AO274"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="67.234375" customWidth="true" bestFit="true"/>
@@ -3188,7 +3241,7 @@
     <col min="25" max="25" width="84.54296875" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="89.12890625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="101.734375" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
@@ -31164,43 +31217,41 @@
         <v>799</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>799</v>
-      </c>
-      <c r="C241" s="2"/>
+        <v>793</v>
+      </c>
+      <c r="C241" t="s" s="2">
+        <v>800</v>
+      </c>
       <c r="D241" t="s" s="2">
-        <v>595</v>
+        <v>78</v>
       </c>
       <c r="E241" s="2"/>
       <c r="F241" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G241" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H241" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I241" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="J241" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K241" t="s" s="2">
-        <v>112</v>
+        <v>801</v>
       </c>
       <c r="L241" t="s" s="2">
-        <v>596</v>
+        <v>802</v>
       </c>
       <c r="M241" t="s" s="2">
-        <v>597</v>
-      </c>
-      <c r="N241" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="O241" t="s" s="2">
-        <v>427</v>
-      </c>
+        <v>803</v>
+      </c>
+      <c r="N241" s="2"/>
+      <c r="O241" s="2"/>
       <c r="P241" t="s" s="2">
         <v>78</v>
       </c>
@@ -31248,7 +31299,7 @@
         <v>78</v>
       </c>
       <c r="AF241" t="s" s="2">
-        <v>598</v>
+        <v>119</v>
       </c>
       <c r="AG241" t="s" s="2">
         <v>79</v>
@@ -31257,7 +31308,7 @@
         <v>80</v>
       </c>
       <c r="AI241" t="s" s="2">
-        <v>78</v>
+        <v>209</v>
       </c>
       <c r="AJ241" t="s" s="2">
         <v>120</v>
@@ -31266,7 +31317,7 @@
         <v>78</v>
       </c>
       <c r="AL241" t="s" s="2">
-        <v>197</v>
+        <v>78</v>
       </c>
       <c r="AM241" t="s" s="2">
         <v>78</v>
@@ -31280,14 +31331,14 @@
     </row>
     <row r="242" hidden="true">
       <c r="A242" t="s" s="2">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C242" s="2"/>
       <c r="D242" t="s" s="2">
-        <v>78</v>
+        <v>595</v>
       </c>
       <c r="E242" s="2"/>
       <c r="F242" t="s" s="2">
@@ -31300,24 +31351,26 @@
         <v>78</v>
       </c>
       <c r="I242" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="J242" t="s" s="2">
         <v>92</v>
       </c>
       <c r="K242" t="s" s="2">
-        <v>237</v>
+        <v>112</v>
       </c>
       <c r="L242" t="s" s="2">
-        <v>801</v>
+        <v>596</v>
       </c>
       <c r="M242" t="s" s="2">
-        <v>802</v>
+        <v>597</v>
       </c>
       <c r="N242" t="s" s="2">
-        <v>803</v>
-      </c>
-      <c r="O242" s="2"/>
+        <v>115</v>
+      </c>
+      <c r="O242" t="s" s="2">
+        <v>427</v>
+      </c>
       <c r="P242" t="s" s="2">
         <v>78</v>
       </c>
@@ -31341,13 +31394,13 @@
         <v>78</v>
       </c>
       <c r="X242" t="s" s="2">
-        <v>163</v>
+        <v>78</v>
       </c>
       <c r="Y242" t="s" s="2">
-        <v>804</v>
+        <v>78</v>
       </c>
       <c r="Z242" t="s" s="2">
-        <v>805</v>
+        <v>78</v>
       </c>
       <c r="AA242" t="s" s="2">
         <v>78</v>
@@ -31365,7 +31418,7 @@
         <v>78</v>
       </c>
       <c r="AF242" t="s" s="2">
-        <v>800</v>
+        <v>598</v>
       </c>
       <c r="AG242" t="s" s="2">
         <v>79</v>
@@ -31377,19 +31430,19 @@
         <v>78</v>
       </c>
       <c r="AJ242" t="s" s="2">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AK242" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL242" t="s" s="2">
-        <v>472</v>
+        <v>197</v>
       </c>
       <c r="AM242" t="s" s="2">
-        <v>472</v>
+        <v>78</v>
       </c>
       <c r="AN242" t="s" s="2">
-        <v>806</v>
+        <v>78</v>
       </c>
       <c r="AO242" t="s" s="2">
         <v>78</v>
@@ -31397,10 +31450,10 @@
     </row>
     <row r="243" hidden="true">
       <c r="A243" t="s" s="2">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B243" t="s" s="2">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="C243" s="2"/>
       <c r="D243" t="s" s="2">
@@ -31411,7 +31464,7 @@
         <v>79</v>
       </c>
       <c r="G243" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H243" t="s" s="2">
         <v>78</v>
@@ -31423,15 +31476,17 @@
         <v>92</v>
       </c>
       <c r="K243" t="s" s="2">
-        <v>261</v>
+        <v>237</v>
       </c>
       <c r="L243" t="s" s="2">
+        <v>806</v>
+      </c>
+      <c r="M243" t="s" s="2">
+        <v>807</v>
+      </c>
+      <c r="N243" t="s" s="2">
         <v>808</v>
       </c>
-      <c r="M243" t="s" s="2">
-        <v>809</v>
-      </c>
-      <c r="N243" s="2"/>
       <c r="O243" s="2"/>
       <c r="P243" t="s" s="2">
         <v>78</v>
@@ -31456,13 +31511,13 @@
         <v>78</v>
       </c>
       <c r="X243" t="s" s="2">
-        <v>78</v>
+        <v>163</v>
       </c>
       <c r="Y243" t="s" s="2">
-        <v>78</v>
+        <v>809</v>
       </c>
       <c r="Z243" t="s" s="2">
-        <v>78</v>
+        <v>810</v>
       </c>
       <c r="AA243" t="s" s="2">
         <v>78</v>
@@ -31480,13 +31535,13 @@
         <v>78</v>
       </c>
       <c r="AF243" t="s" s="2">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="AG243" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH243" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AI243" t="s" s="2">
         <v>78</v>
@@ -31498,13 +31553,13 @@
         <v>78</v>
       </c>
       <c r="AL243" t="s" s="2">
-        <v>543</v>
+        <v>472</v>
       </c>
       <c r="AM243" t="s" s="2">
-        <v>543</v>
+        <v>472</v>
       </c>
       <c r="AN243" t="s" s="2">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="AO243" t="s" s="2">
         <v>78</v>
@@ -31512,10 +31567,10 @@
     </row>
     <row r="244" hidden="true">
       <c r="A244" t="s" s="2">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="B244" t="s" s="2">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="C244" s="2"/>
       <c r="D244" t="s" s="2">
@@ -31538,7 +31593,7 @@
         <v>92</v>
       </c>
       <c r="K244" t="s" s="2">
-        <v>812</v>
+        <v>261</v>
       </c>
       <c r="L244" t="s" s="2">
         <v>813</v>
@@ -31595,13 +31650,13 @@
         <v>78</v>
       </c>
       <c r="AF244" t="s" s="2">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="AG244" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH244" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AI244" t="s" s="2">
         <v>78</v>
@@ -31613,13 +31668,13 @@
         <v>78</v>
       </c>
       <c r="AL244" t="s" s="2">
+        <v>543</v>
+      </c>
+      <c r="AM244" t="s" s="2">
+        <v>543</v>
+      </c>
+      <c r="AN244" t="s" s="2">
         <v>815</v>
-      </c>
-      <c r="AM244" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="AN244" t="s" s="2">
-        <v>78</v>
       </c>
       <c r="AO244" t="s" s="2">
         <v>78</v>
@@ -31630,17 +31685,15 @@
         <v>816</v>
       </c>
       <c r="B245" t="s" s="2">
-        <v>783</v>
-      </c>
-      <c r="C245" t="s" s="2">
-        <v>817</v>
-      </c>
+        <v>816</v>
+      </c>
+      <c r="C245" s="2"/>
       <c r="D245" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E245" s="2"/>
       <c r="F245" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G245" t="s" s="2">
         <v>91</v>
@@ -31655,20 +31708,16 @@
         <v>92</v>
       </c>
       <c r="K245" t="s" s="2">
-        <v>582</v>
+        <v>817</v>
       </c>
       <c r="L245" t="s" s="2">
         <v>818</v>
       </c>
       <c r="M245" t="s" s="2">
-        <v>785</v>
-      </c>
-      <c r="N245" t="s" s="2">
-        <v>786</v>
-      </c>
-      <c r="O245" t="s" s="2">
-        <v>787</v>
-      </c>
+        <v>819</v>
+      </c>
+      <c r="N245" s="2"/>
+      <c r="O245" s="2"/>
       <c r="P245" t="s" s="2">
         <v>78</v>
       </c>
@@ -31716,7 +31765,7 @@
         <v>78</v>
       </c>
       <c r="AF245" t="s" s="2">
-        <v>783</v>
+        <v>816</v>
       </c>
       <c r="AG245" t="s" s="2">
         <v>79</v>
@@ -31734,13 +31783,13 @@
         <v>78</v>
       </c>
       <c r="AL245" t="s" s="2">
-        <v>789</v>
+        <v>820</v>
       </c>
       <c r="AM245" t="s" s="2">
-        <v>790</v>
+        <v>109</v>
       </c>
       <c r="AN245" t="s" s="2">
-        <v>791</v>
+        <v>78</v>
       </c>
       <c r="AO245" t="s" s="2">
         <v>78</v>
@@ -31748,18 +31797,20 @@
     </row>
     <row r="246" hidden="true">
       <c r="A246" t="s" s="2">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="B246" t="s" s="2">
-        <v>792</v>
-      </c>
-      <c r="C246" s="2"/>
+        <v>783</v>
+      </c>
+      <c r="C246" t="s" s="2">
+        <v>822</v>
+      </c>
       <c r="D246" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E246" s="2"/>
       <c r="F246" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G246" t="s" s="2">
         <v>91</v>
@@ -31771,19 +31822,23 @@
         <v>78</v>
       </c>
       <c r="J246" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K246" t="s" s="2">
-        <v>105</v>
+        <v>582</v>
       </c>
       <c r="L246" t="s" s="2">
-        <v>106</v>
+        <v>823</v>
       </c>
       <c r="M246" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="N246" s="2"/>
-      <c r="O246" s="2"/>
+        <v>785</v>
+      </c>
+      <c r="N246" t="s" s="2">
+        <v>786</v>
+      </c>
+      <c r="O246" t="s" s="2">
+        <v>787</v>
+      </c>
       <c r="P246" t="s" s="2">
         <v>78</v>
       </c>
@@ -31831,31 +31886,31 @@
         <v>78</v>
       </c>
       <c r="AF246" t="s" s="2">
-        <v>108</v>
+        <v>783</v>
       </c>
       <c r="AG246" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH246" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AI246" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ246" t="s" s="2">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="AK246" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL246" t="s" s="2">
-        <v>109</v>
+        <v>789</v>
       </c>
       <c r="AM246" t="s" s="2">
-        <v>78</v>
+        <v>790</v>
       </c>
       <c r="AN246" t="s" s="2">
-        <v>78</v>
+        <v>791</v>
       </c>
       <c r="AO246" t="s" s="2">
         <v>78</v>
@@ -31863,10 +31918,10 @@
     </row>
     <row r="247" hidden="true">
       <c r="A247" t="s" s="2">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="B247" t="s" s="2">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="C247" s="2"/>
       <c r="D247" t="s" s="2">
@@ -31874,10 +31929,10 @@
       </c>
       <c r="E247" s="2"/>
       <c r="F247" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G247" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H247" t="s" s="2">
         <v>78</v>
@@ -31889,13 +31944,13 @@
         <v>78</v>
       </c>
       <c r="K247" t="s" s="2">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="L247" t="s" s="2">
-        <v>199</v>
+        <v>106</v>
       </c>
       <c r="M247" t="s" s="2">
-        <v>200</v>
+        <v>107</v>
       </c>
       <c r="N247" s="2"/>
       <c r="O247" s="2"/>
@@ -31934,35 +31989,37 @@
         <v>78</v>
       </c>
       <c r="AB247" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AC247" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="AC247" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="AD247" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE247" t="s" s="2">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="AF247" t="s" s="2">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="AG247" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH247" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AI247" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ247" t="s" s="2">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="AK247" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL247" t="s" s="2">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="AM247" t="s" s="2">
         <v>78</v>
@@ -31976,23 +32033,21 @@
     </row>
     <row r="248" hidden="true">
       <c r="A248" t="s" s="2">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="B248" t="s" s="2">
         <v>793</v>
       </c>
-      <c r="C248" t="s" s="2">
-        <v>795</v>
-      </c>
+      <c r="C248" s="2"/>
       <c r="D248" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E248" s="2"/>
       <c r="F248" t="s" s="2">
-        <v>91</v>
+        <v>283</v>
       </c>
       <c r="G248" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H248" t="s" s="2">
         <v>78</v>
@@ -32004,13 +32059,13 @@
         <v>78</v>
       </c>
       <c r="K248" t="s" s="2">
-        <v>796</v>
+        <v>112</v>
       </c>
       <c r="L248" t="s" s="2">
-        <v>822</v>
+        <v>199</v>
       </c>
       <c r="M248" t="s" s="2">
-        <v>798</v>
+        <v>200</v>
       </c>
       <c r="N248" s="2"/>
       <c r="O248" s="2"/>
@@ -32049,16 +32104,14 @@
         <v>78</v>
       </c>
       <c r="AB248" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC248" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="AC248" s="2"/>
       <c r="AD248" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE248" t="s" s="2">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="AF248" t="s" s="2">
         <v>119</v>
@@ -32070,7 +32123,7 @@
         <v>80</v>
       </c>
       <c r="AI248" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ248" t="s" s="2">
         <v>120</v>
@@ -32093,46 +32146,44 @@
     </row>
     <row r="249" hidden="true">
       <c r="A249" t="s" s="2">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="B249" t="s" s="2">
-        <v>799</v>
-      </c>
-      <c r="C249" s="2"/>
+        <v>793</v>
+      </c>
+      <c r="C249" t="s" s="2">
+        <v>795</v>
+      </c>
       <c r="D249" t="s" s="2">
-        <v>595</v>
+        <v>78</v>
       </c>
       <c r="E249" s="2"/>
       <c r="F249" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G249" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H249" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I249" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="J249" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K249" t="s" s="2">
-        <v>112</v>
+        <v>796</v>
       </c>
       <c r="L249" t="s" s="2">
-        <v>596</v>
+        <v>827</v>
       </c>
       <c r="M249" t="s" s="2">
-        <v>597</v>
-      </c>
-      <c r="N249" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="O249" t="s" s="2">
-        <v>427</v>
-      </c>
+        <v>798</v>
+      </c>
+      <c r="N249" s="2"/>
+      <c r="O249" s="2"/>
       <c r="P249" t="s" s="2">
         <v>78</v>
       </c>
@@ -32180,7 +32231,7 @@
         <v>78</v>
       </c>
       <c r="AF249" t="s" s="2">
-        <v>598</v>
+        <v>119</v>
       </c>
       <c r="AG249" t="s" s="2">
         <v>79</v>
@@ -32189,7 +32240,7 @@
         <v>80</v>
       </c>
       <c r="AI249" t="s" s="2">
-        <v>78</v>
+        <v>209</v>
       </c>
       <c r="AJ249" t="s" s="2">
         <v>120</v>
@@ -32198,7 +32249,7 @@
         <v>78</v>
       </c>
       <c r="AL249" t="s" s="2">
-        <v>197</v>
+        <v>78</v>
       </c>
       <c r="AM249" t="s" s="2">
         <v>78</v>
@@ -32212,21 +32263,23 @@
     </row>
     <row r="250" hidden="true">
       <c r="A250" t="s" s="2">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="B250" t="s" s="2">
+        <v>793</v>
+      </c>
+      <c r="C250" t="s" s="2">
         <v>800</v>
       </c>
-      <c r="C250" s="2"/>
       <c r="D250" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E250" s="2"/>
       <c r="F250" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G250" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H250" t="s" s="2">
         <v>78</v>
@@ -32235,20 +32288,18 @@
         <v>78</v>
       </c>
       <c r="J250" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K250" t="s" s="2">
-        <v>237</v>
+        <v>801</v>
       </c>
       <c r="L250" t="s" s="2">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="M250" t="s" s="2">
-        <v>802</v>
-      </c>
-      <c r="N250" t="s" s="2">
         <v>803</v>
       </c>
+      <c r="N250" s="2"/>
       <c r="O250" s="2"/>
       <c r="P250" t="s" s="2">
         <v>78</v>
@@ -32273,13 +32324,13 @@
         <v>78</v>
       </c>
       <c r="X250" t="s" s="2">
-        <v>163</v>
+        <v>78</v>
       </c>
       <c r="Y250" t="s" s="2">
-        <v>804</v>
+        <v>78</v>
       </c>
       <c r="Z250" t="s" s="2">
-        <v>805</v>
+        <v>78</v>
       </c>
       <c r="AA250" t="s" s="2">
         <v>78</v>
@@ -32297,7 +32348,7 @@
         <v>78</v>
       </c>
       <c r="AF250" t="s" s="2">
-        <v>800</v>
+        <v>119</v>
       </c>
       <c r="AG250" t="s" s="2">
         <v>79</v>
@@ -32306,22 +32357,22 @@
         <v>80</v>
       </c>
       <c r="AI250" t="s" s="2">
-        <v>78</v>
+        <v>209</v>
       </c>
       <c r="AJ250" t="s" s="2">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AK250" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL250" t="s" s="2">
-        <v>472</v>
+        <v>78</v>
       </c>
       <c r="AM250" t="s" s="2">
-        <v>472</v>
+        <v>78</v>
       </c>
       <c r="AN250" t="s" s="2">
-        <v>806</v>
+        <v>78</v>
       </c>
       <c r="AO250" t="s" s="2">
         <v>78</v>
@@ -32329,10 +32380,10 @@
     </row>
     <row r="251" hidden="true">
       <c r="A251" t="s" s="2">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="B251" t="s" s="2">
-        <v>807</v>
+        <v>830</v>
       </c>
       <c r="C251" s="2"/>
       <c r="D251" t="s" s="2">
@@ -32340,7 +32391,7 @@
       </c>
       <c r="E251" s="2"/>
       <c r="F251" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G251" t="s" s="2">
         <v>91</v>
@@ -32352,16 +32403,16 @@
         <v>78</v>
       </c>
       <c r="J251" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K251" t="s" s="2">
-        <v>261</v>
+        <v>105</v>
       </c>
       <c r="L251" t="s" s="2">
-        <v>826</v>
+        <v>106</v>
       </c>
       <c r="M251" t="s" s="2">
-        <v>809</v>
+        <v>107</v>
       </c>
       <c r="N251" s="2"/>
       <c r="O251" s="2"/>
@@ -32412,7 +32463,7 @@
         <v>78</v>
       </c>
       <c r="AF251" t="s" s="2">
-        <v>807</v>
+        <v>108</v>
       </c>
       <c r="AG251" t="s" s="2">
         <v>79</v>
@@ -32424,19 +32475,19 @@
         <v>78</v>
       </c>
       <c r="AJ251" t="s" s="2">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="AK251" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL251" t="s" s="2">
-        <v>543</v>
+        <v>109</v>
       </c>
       <c r="AM251" t="s" s="2">
-        <v>543</v>
+        <v>78</v>
       </c>
       <c r="AN251" t="s" s="2">
-        <v>810</v>
+        <v>78</v>
       </c>
       <c r="AO251" t="s" s="2">
         <v>78</v>
@@ -32444,10 +32495,10 @@
     </row>
     <row r="252" hidden="true">
       <c r="A252" t="s" s="2">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="B252" t="s" s="2">
-        <v>811</v>
+        <v>832</v>
       </c>
       <c r="C252" s="2"/>
       <c r="D252" t="s" s="2">
@@ -32458,7 +32509,7 @@
         <v>79</v>
       </c>
       <c r="G252" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="H252" t="s" s="2">
         <v>78</v>
@@ -32467,16 +32518,16 @@
         <v>78</v>
       </c>
       <c r="J252" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K252" t="s" s="2">
-        <v>812</v>
+        <v>112</v>
       </c>
       <c r="L252" t="s" s="2">
-        <v>813</v>
+        <v>199</v>
       </c>
       <c r="M252" t="s" s="2">
-        <v>814</v>
+        <v>200</v>
       </c>
       <c r="N252" s="2"/>
       <c r="O252" s="2"/>
@@ -32515,19 +32566,19 @@
         <v>78</v>
       </c>
       <c r="AB252" t="s" s="2">
-        <v>78</v>
+        <v>116</v>
       </c>
       <c r="AC252" t="s" s="2">
-        <v>78</v>
+        <v>117</v>
       </c>
       <c r="AD252" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE252" t="s" s="2">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="AF252" t="s" s="2">
-        <v>811</v>
+        <v>119</v>
       </c>
       <c r="AG252" t="s" s="2">
         <v>79</v>
@@ -32539,16 +32590,16 @@
         <v>78</v>
       </c>
       <c r="AJ252" t="s" s="2">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AK252" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL252" t="s" s="2">
-        <v>815</v>
+        <v>78</v>
       </c>
       <c r="AM252" t="s" s="2">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="AN252" t="s" s="2">
         <v>78</v>
@@ -32557,12 +32608,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="253">
+    <row r="253" hidden="true">
       <c r="A253" t="s" s="2">
-        <v>828</v>
+        <v>833</v>
       </c>
       <c r="B253" t="s" s="2">
-        <v>828</v>
+        <v>834</v>
       </c>
       <c r="C253" s="2"/>
       <c r="D253" t="s" s="2">
@@ -32573,10 +32624,10 @@
         <v>91</v>
       </c>
       <c r="G253" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H253" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="I253" t="s" s="2">
         <v>78</v>
@@ -32585,22 +32636,24 @@
         <v>78</v>
       </c>
       <c r="K253" t="s" s="2">
-        <v>582</v>
+        <v>133</v>
       </c>
       <c r="L253" t="s" s="2">
-        <v>829</v>
+        <v>231</v>
       </c>
       <c r="M253" t="s" s="2">
-        <v>830</v>
-      </c>
-      <c r="N253" s="2"/>
+        <v>232</v>
+      </c>
+      <c r="N253" t="s" s="2">
+        <v>233</v>
+      </c>
       <c r="O253" s="2"/>
       <c r="P253" t="s" s="2">
         <v>78</v>
       </c>
       <c r="Q253" s="2"/>
       <c r="R253" t="s" s="2">
-        <v>78</v>
+        <v>835</v>
       </c>
       <c r="S253" t="s" s="2">
         <v>78</v>
@@ -32642,28 +32695,28 @@
         <v>78</v>
       </c>
       <c r="AF253" t="s" s="2">
-        <v>828</v>
+        <v>234</v>
       </c>
       <c r="AG253" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="AH253" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AI253" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ253" t="s" s="2">
-        <v>831</v>
+        <v>78</v>
       </c>
       <c r="AK253" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL253" t="s" s="2">
-        <v>832</v>
+        <v>197</v>
       </c>
       <c r="AM253" t="s" s="2">
-        <v>833</v>
+        <v>78</v>
       </c>
       <c r="AN253" t="s" s="2">
         <v>78</v>
@@ -32674,10 +32727,10 @@
     </row>
     <row r="254" hidden="true">
       <c r="A254" t="s" s="2">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="B254" t="s" s="2">
-        <v>834</v>
+        <v>837</v>
       </c>
       <c r="C254" s="2"/>
       <c r="D254" t="s" s="2">
@@ -32685,7 +32738,7 @@
       </c>
       <c r="E254" s="2"/>
       <c r="F254" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G254" t="s" s="2">
         <v>91</v>
@@ -32700,13 +32753,13 @@
         <v>78</v>
       </c>
       <c r="K254" t="s" s="2">
-        <v>105</v>
+        <v>838</v>
       </c>
       <c r="L254" t="s" s="2">
-        <v>106</v>
+        <v>238</v>
       </c>
       <c r="M254" t="s" s="2">
-        <v>107</v>
+        <v>239</v>
       </c>
       <c r="N254" s="2"/>
       <c r="O254" s="2"/>
@@ -32718,7 +32771,7 @@
         <v>78</v>
       </c>
       <c r="S254" t="s" s="2">
-        <v>78</v>
+        <v>839</v>
       </c>
       <c r="T254" t="s" s="2">
         <v>78</v>
@@ -32757,7 +32810,7 @@
         <v>78</v>
       </c>
       <c r="AF254" t="s" s="2">
-        <v>108</v>
+        <v>242</v>
       </c>
       <c r="AG254" t="s" s="2">
         <v>79</v>
@@ -32769,13 +32822,13 @@
         <v>78</v>
       </c>
       <c r="AJ254" t="s" s="2">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="AK254" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL254" t="s" s="2">
-        <v>109</v>
+        <v>197</v>
       </c>
       <c r="AM254" t="s" s="2">
         <v>78</v>
@@ -32789,14 +32842,14 @@
     </row>
     <row r="255" hidden="true">
       <c r="A255" t="s" s="2">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B255" t="s" s="2">
-        <v>835</v>
+        <v>804</v>
       </c>
       <c r="C255" s="2"/>
       <c r="D255" t="s" s="2">
-        <v>78</v>
+        <v>595</v>
       </c>
       <c r="E255" s="2"/>
       <c r="F255" t="s" s="2">
@@ -32809,22 +32862,26 @@
         <v>78</v>
       </c>
       <c r="I255" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="J255" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K255" t="s" s="2">
         <v>112</v>
       </c>
       <c r="L255" t="s" s="2">
-        <v>199</v>
+        <v>596</v>
       </c>
       <c r="M255" t="s" s="2">
-        <v>200</v>
-      </c>
-      <c r="N255" s="2"/>
-      <c r="O255" s="2"/>
+        <v>597</v>
+      </c>
+      <c r="N255" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="O255" t="s" s="2">
+        <v>427</v>
+      </c>
       <c r="P255" t="s" s="2">
         <v>78</v>
       </c>
@@ -32860,17 +32917,19 @@
         <v>78</v>
       </c>
       <c r="AB255" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="AC255" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="AC255" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="AD255" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE255" t="s" s="2">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="AF255" t="s" s="2">
-        <v>119</v>
+        <v>598</v>
       </c>
       <c r="AG255" t="s" s="2">
         <v>79</v>
@@ -32888,7 +32947,7 @@
         <v>78</v>
       </c>
       <c r="AL255" t="s" s="2">
-        <v>78</v>
+        <v>197</v>
       </c>
       <c r="AM255" t="s" s="2">
         <v>78</v>
@@ -32902,14 +32961,12 @@
     </row>
     <row r="256" hidden="true">
       <c r="A256" t="s" s="2">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="B256" t="s" s="2">
-        <v>835</v>
-      </c>
-      <c r="C256" t="s" s="2">
-        <v>407</v>
-      </c>
+        <v>805</v>
+      </c>
+      <c r="C256" s="2"/>
       <c r="D256" t="s" s="2">
         <v>78</v>
       </c>
@@ -32918,7 +32975,7 @@
         <v>79</v>
       </c>
       <c r="G256" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H256" t="s" s="2">
         <v>78</v>
@@ -32927,18 +32984,20 @@
         <v>78</v>
       </c>
       <c r="J256" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K256" t="s" s="2">
-        <v>409</v>
+        <v>237</v>
       </c>
       <c r="L256" t="s" s="2">
-        <v>837</v>
+        <v>806</v>
       </c>
       <c r="M256" t="s" s="2">
-        <v>410</v>
-      </c>
-      <c r="N256" s="2"/>
+        <v>807</v>
+      </c>
+      <c r="N256" t="s" s="2">
+        <v>808</v>
+      </c>
       <c r="O256" s="2"/>
       <c r="P256" t="s" s="2">
         <v>78</v>
@@ -32963,13 +33022,13 @@
         <v>78</v>
       </c>
       <c r="X256" t="s" s="2">
-        <v>78</v>
+        <v>163</v>
       </c>
       <c r="Y256" t="s" s="2">
-        <v>78</v>
+        <v>809</v>
       </c>
       <c r="Z256" t="s" s="2">
-        <v>78</v>
+        <v>810</v>
       </c>
       <c r="AA256" t="s" s="2">
         <v>78</v>
@@ -32987,7 +33046,7 @@
         <v>78</v>
       </c>
       <c r="AF256" t="s" s="2">
-        <v>119</v>
+        <v>805</v>
       </c>
       <c r="AG256" t="s" s="2">
         <v>79</v>
@@ -32996,22 +33055,22 @@
         <v>80</v>
       </c>
       <c r="AI256" t="s" s="2">
-        <v>209</v>
+        <v>78</v>
       </c>
       <c r="AJ256" t="s" s="2">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="AK256" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL256" t="s" s="2">
-        <v>78</v>
+        <v>472</v>
       </c>
       <c r="AM256" t="s" s="2">
-        <v>78</v>
+        <v>472</v>
       </c>
       <c r="AN256" t="s" s="2">
-        <v>78</v>
+        <v>811</v>
       </c>
       <c r="AO256" t="s" s="2">
         <v>78</v>
@@ -33019,23 +33078,21 @@
     </row>
     <row r="257" hidden="true">
       <c r="A257" t="s" s="2">
-        <v>838</v>
+        <v>842</v>
       </c>
       <c r="B257" t="s" s="2">
-        <v>835</v>
-      </c>
-      <c r="C257" t="s" s="2">
-        <v>839</v>
-      </c>
+        <v>812</v>
+      </c>
+      <c r="C257" s="2"/>
       <c r="D257" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E257" s="2"/>
       <c r="F257" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G257" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H257" t="s" s="2">
         <v>78</v>
@@ -33044,20 +33101,18 @@
         <v>78</v>
       </c>
       <c r="J257" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K257" t="s" s="2">
-        <v>840</v>
+        <v>261</v>
       </c>
       <c r="L257" t="s" s="2">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="M257" t="s" s="2">
-        <v>842</v>
-      </c>
-      <c r="N257" t="s" s="2">
-        <v>843</v>
-      </c>
+        <v>814</v>
+      </c>
+      <c r="N257" s="2"/>
       <c r="O257" s="2"/>
       <c r="P257" t="s" s="2">
         <v>78</v>
@@ -33106,31 +33161,31 @@
         <v>78</v>
       </c>
       <c r="AF257" t="s" s="2">
-        <v>119</v>
+        <v>812</v>
       </c>
       <c r="AG257" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH257" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AI257" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ257" t="s" s="2">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="AK257" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL257" t="s" s="2">
-        <v>78</v>
+        <v>543</v>
       </c>
       <c r="AM257" t="s" s="2">
-        <v>78</v>
+        <v>543</v>
       </c>
       <c r="AN257" t="s" s="2">
-        <v>78</v>
+        <v>815</v>
       </c>
       <c r="AO257" t="s" s="2">
         <v>78</v>
@@ -33141,43 +33196,39 @@
         <v>844</v>
       </c>
       <c r="B258" t="s" s="2">
-        <v>844</v>
+        <v>816</v>
       </c>
       <c r="C258" s="2"/>
       <c r="D258" t="s" s="2">
-        <v>595</v>
+        <v>78</v>
       </c>
       <c r="E258" s="2"/>
       <c r="F258" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G258" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H258" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I258" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="J258" t="s" s="2">
         <v>92</v>
       </c>
       <c r="K258" t="s" s="2">
-        <v>112</v>
+        <v>817</v>
       </c>
       <c r="L258" t="s" s="2">
-        <v>596</v>
+        <v>818</v>
       </c>
       <c r="M258" t="s" s="2">
-        <v>597</v>
-      </c>
-      <c r="N258" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="O258" t="s" s="2">
-        <v>427</v>
-      </c>
+        <v>819</v>
+      </c>
+      <c r="N258" s="2"/>
+      <c r="O258" s="2"/>
       <c r="P258" t="s" s="2">
         <v>78</v>
       </c>
@@ -33225,7 +33276,7 @@
         <v>78</v>
       </c>
       <c r="AF258" t="s" s="2">
-        <v>598</v>
+        <v>816</v>
       </c>
       <c r="AG258" t="s" s="2">
         <v>79</v>
@@ -33237,16 +33288,16 @@
         <v>78</v>
       </c>
       <c r="AJ258" t="s" s="2">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="AK258" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL258" t="s" s="2">
-        <v>197</v>
+        <v>820</v>
       </c>
       <c r="AM258" t="s" s="2">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="AN258" t="s" s="2">
         <v>78</v>
@@ -33264,14 +33315,14 @@
       </c>
       <c r="C259" s="2"/>
       <c r="D259" t="s" s="2">
-        <v>846</v>
+        <v>78</v>
       </c>
       <c r="E259" s="2"/>
       <c r="F259" t="s" s="2">
         <v>91</v>
       </c>
       <c r="G259" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H259" t="s" s="2">
         <v>92</v>
@@ -33283,20 +33334,16 @@
         <v>78</v>
       </c>
       <c r="K259" t="s" s="2">
-        <v>105</v>
+        <v>582</v>
       </c>
       <c r="L259" t="s" s="2">
+        <v>846</v>
+      </c>
+      <c r="M259" t="s" s="2">
         <v>847</v>
       </c>
-      <c r="M259" t="s" s="2">
-        <v>848</v>
-      </c>
-      <c r="N259" t="s" s="2">
-        <v>849</v>
-      </c>
-      <c r="O259" t="s" s="2">
-        <v>850</v>
-      </c>
+      <c r="N259" s="2"/>
+      <c r="O259" s="2"/>
       <c r="P259" t="s" s="2">
         <v>78</v>
       </c>
@@ -33350,22 +33397,22 @@
         <v>79</v>
       </c>
       <c r="AH259" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AI259" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ259" t="s" s="2">
-        <v>103</v>
+        <v>848</v>
       </c>
       <c r="AK259" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL259" t="s" s="2">
-        <v>570</v>
+        <v>849</v>
       </c>
       <c r="AM259" t="s" s="2">
-        <v>571</v>
+        <v>850</v>
       </c>
       <c r="AN259" t="s" s="2">
         <v>78</v>
@@ -33374,7 +33421,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="260">
+    <row r="260" hidden="true">
       <c r="A260" t="s" s="2">
         <v>851</v>
       </c>
@@ -33387,13 +33434,13 @@
       </c>
       <c r="E260" s="2"/>
       <c r="F260" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G260" t="s" s="2">
         <v>91</v>
       </c>
       <c r="H260" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="I260" t="s" s="2">
         <v>78</v>
@@ -33402,20 +33449,16 @@
         <v>78</v>
       </c>
       <c r="K260" t="s" s="2">
-        <v>237</v>
+        <v>105</v>
       </c>
       <c r="L260" t="s" s="2">
-        <v>852</v>
+        <v>106</v>
       </c>
       <c r="M260" t="s" s="2">
-        <v>853</v>
-      </c>
-      <c r="N260" t="s" s="2">
-        <v>854</v>
-      </c>
-      <c r="O260" t="s" s="2">
-        <v>855</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="N260" s="2"/>
+      <c r="O260" s="2"/>
       <c r="P260" t="s" s="2">
         <v>78</v>
       </c>
@@ -33439,11 +33482,13 @@
         <v>78</v>
       </c>
       <c r="X260" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="Y260" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="Y260" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="Z260" t="s" s="2">
-        <v>856</v>
+        <v>78</v>
       </c>
       <c r="AA260" t="s" s="2">
         <v>78</v>
@@ -33461,7 +33506,7 @@
         <v>78</v>
       </c>
       <c r="AF260" t="s" s="2">
-        <v>851</v>
+        <v>108</v>
       </c>
       <c r="AG260" t="s" s="2">
         <v>79</v>
@@ -33473,16 +33518,16 @@
         <v>78</v>
       </c>
       <c r="AJ260" t="s" s="2">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="AK260" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL260" t="s" s="2">
-        <v>471</v>
+        <v>109</v>
       </c>
       <c r="AM260" t="s" s="2">
-        <v>472</v>
+        <v>78</v>
       </c>
       <c r="AN260" t="s" s="2">
         <v>78</v>
@@ -33493,10 +33538,10 @@
     </row>
     <row r="261" hidden="true">
       <c r="A261" t="s" s="2">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="B261" t="s" s="2">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="C261" s="2"/>
       <c r="D261" t="s" s="2">
@@ -33519,18 +33564,16 @@
         <v>78</v>
       </c>
       <c r="K261" t="s" s="2">
-        <v>858</v>
+        <v>112</v>
       </c>
       <c r="L261" t="s" s="2">
-        <v>859</v>
+        <v>199</v>
       </c>
       <c r="M261" t="s" s="2">
-        <v>860</v>
+        <v>200</v>
       </c>
       <c r="N261" s="2"/>
-      <c r="O261" t="s" s="2">
-        <v>550</v>
-      </c>
+      <c r="O261" s="2"/>
       <c r="P261" t="s" s="2">
         <v>78</v>
       </c>
@@ -33566,19 +33609,17 @@
         <v>78</v>
       </c>
       <c r="AB261" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC261" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="AC261" s="2"/>
       <c r="AD261" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE261" t="s" s="2">
-        <v>78</v>
+        <v>118</v>
       </c>
       <c r="AF261" t="s" s="2">
-        <v>857</v>
+        <v>119</v>
       </c>
       <c r="AG261" t="s" s="2">
         <v>79</v>
@@ -33590,32 +33631,34 @@
         <v>78</v>
       </c>
       <c r="AJ261" t="s" s="2">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AK261" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL261" t="s" s="2">
-        <v>552</v>
+        <v>78</v>
       </c>
       <c r="AM261" t="s" s="2">
-        <v>553</v>
+        <v>78</v>
       </c>
       <c r="AN261" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AO261" t="s" s="2">
-        <v>555</v>
+        <v>78</v>
       </c>
     </row>
     <row r="262" hidden="true">
       <c r="A262" t="s" s="2">
-        <v>861</v>
+        <v>853</v>
       </c>
       <c r="B262" t="s" s="2">
-        <v>861</v>
-      </c>
-      <c r="C262" s="2"/>
+        <v>852</v>
+      </c>
+      <c r="C262" t="s" s="2">
+        <v>407</v>
+      </c>
       <c r="D262" t="s" s="2">
         <v>78</v>
       </c>
@@ -33636,17 +33679,15 @@
         <v>78</v>
       </c>
       <c r="K262" t="s" s="2">
-        <v>812</v>
+        <v>409</v>
       </c>
       <c r="L262" t="s" s="2">
-        <v>862</v>
+        <v>854</v>
       </c>
       <c r="M262" t="s" s="2">
-        <v>863</v>
-      </c>
-      <c r="N262" t="s" s="2">
-        <v>864</v>
-      </c>
+        <v>410</v>
+      </c>
+      <c r="N262" s="2"/>
       <c r="O262" s="2"/>
       <c r="P262" t="s" s="2">
         <v>78</v>
@@ -33695,19 +33736,19 @@
         <v>78</v>
       </c>
       <c r="AF262" t="s" s="2">
-        <v>861</v>
+        <v>119</v>
       </c>
       <c r="AG262" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH262" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AI262" t="s" s="2">
-        <v>78</v>
+        <v>209</v>
       </c>
       <c r="AJ262" t="s" s="2">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AK262" t="s" s="2">
         <v>78</v>
@@ -33716,7 +33757,7 @@
         <v>78</v>
       </c>
       <c r="AM262" t="s" s="2">
-        <v>865</v>
+        <v>78</v>
       </c>
       <c r="AN262" t="s" s="2">
         <v>78</v>
@@ -33725,26 +33766,28 @@
         <v>78</v>
       </c>
     </row>
-    <row r="263">
+    <row r="263" hidden="true">
       <c r="A263" t="s" s="2">
-        <v>866</v>
+        <v>855</v>
       </c>
       <c r="B263" t="s" s="2">
-        <v>866</v>
-      </c>
-      <c r="C263" s="2"/>
+        <v>852</v>
+      </c>
+      <c r="C263" t="s" s="2">
+        <v>856</v>
+      </c>
       <c r="D263" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E263" s="2"/>
       <c r="F263" t="s" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G263" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H263" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="I263" t="s" s="2">
         <v>78</v>
@@ -33753,16 +33796,16 @@
         <v>78</v>
       </c>
       <c r="K263" t="s" s="2">
-        <v>184</v>
+        <v>857</v>
       </c>
       <c r="L263" t="s" s="2">
-        <v>867</v>
+        <v>858</v>
       </c>
       <c r="M263" t="s" s="2">
-        <v>868</v>
+        <v>859</v>
       </c>
       <c r="N263" t="s" s="2">
-        <v>869</v>
+        <v>860</v>
       </c>
       <c r="O263" s="2"/>
       <c r="P263" t="s" s="2">
@@ -33812,28 +33855,28 @@
         <v>78</v>
       </c>
       <c r="AF263" t="s" s="2">
-        <v>866</v>
+        <v>119</v>
       </c>
       <c r="AG263" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH263" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AI263" t="s" s="2">
-        <v>870</v>
+        <v>78</v>
       </c>
       <c r="AJ263" t="s" s="2">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AK263" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL263" t="s" s="2">
-        <v>871</v>
+        <v>78</v>
       </c>
       <c r="AM263" t="s" s="2">
-        <v>871</v>
+        <v>78</v>
       </c>
       <c r="AN263" t="s" s="2">
         <v>78</v>
@@ -33844,45 +33887,45 @@
     </row>
     <row r="264" hidden="true">
       <c r="A264" t="s" s="2">
-        <v>872</v>
+        <v>861</v>
       </c>
       <c r="B264" t="s" s="2">
-        <v>872</v>
+        <v>861</v>
       </c>
       <c r="C264" s="2"/>
       <c r="D264" t="s" s="2">
-        <v>78</v>
+        <v>595</v>
       </c>
       <c r="E264" s="2"/>
       <c r="F264" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G264" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H264" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I264" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="J264" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K264" t="s" s="2">
-        <v>173</v>
+        <v>112</v>
       </c>
       <c r="L264" t="s" s="2">
-        <v>873</v>
+        <v>596</v>
       </c>
       <c r="M264" t="s" s="2">
-        <v>874</v>
+        <v>597</v>
       </c>
       <c r="N264" t="s" s="2">
-        <v>875</v>
+        <v>115</v>
       </c>
       <c r="O264" t="s" s="2">
-        <v>876</v>
+        <v>427</v>
       </c>
       <c r="P264" t="s" s="2">
         <v>78</v>
@@ -33907,13 +33950,13 @@
         <v>78</v>
       </c>
       <c r="X264" t="s" s="2">
-        <v>327</v>
+        <v>78</v>
       </c>
       <c r="Y264" t="s" s="2">
-        <v>877</v>
+        <v>78</v>
       </c>
       <c r="Z264" t="s" s="2">
-        <v>878</v>
+        <v>78</v>
       </c>
       <c r="AA264" t="s" s="2">
         <v>78</v>
@@ -33931,56 +33974,56 @@
         <v>78</v>
       </c>
       <c r="AF264" t="s" s="2">
-        <v>872</v>
+        <v>598</v>
       </c>
       <c r="AG264" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH264" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AI264" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ264" t="s" s="2">
-        <v>103</v>
+        <v>120</v>
       </c>
       <c r="AK264" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL264" t="s" s="2">
-        <v>879</v>
+        <v>197</v>
       </c>
       <c r="AM264" t="s" s="2">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="AN264" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AO264" t="s" s="2">
-        <v>474</v>
+        <v>78</v>
       </c>
     </row>
-    <row r="265" hidden="true">
+    <row r="265">
       <c r="A265" t="s" s="2">
-        <v>880</v>
+        <v>862</v>
       </c>
       <c r="B265" t="s" s="2">
-        <v>880</v>
+        <v>862</v>
       </c>
       <c r="C265" s="2"/>
       <c r="D265" t="s" s="2">
-        <v>78</v>
+        <v>863</v>
       </c>
       <c r="E265" s="2"/>
       <c r="F265" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G265" t="s" s="2">
         <v>91</v>
       </c>
       <c r="H265" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="I265" t="s" s="2">
         <v>78</v>
@@ -33989,19 +34032,19 @@
         <v>78</v>
       </c>
       <c r="K265" t="s" s="2">
-        <v>237</v>
+        <v>105</v>
       </c>
       <c r="L265" t="s" s="2">
-        <v>881</v>
+        <v>864</v>
       </c>
       <c r="M265" t="s" s="2">
-        <v>882</v>
+        <v>865</v>
       </c>
       <c r="N265" t="s" s="2">
-        <v>883</v>
+        <v>866</v>
       </c>
       <c r="O265" t="s" s="2">
-        <v>884</v>
+        <v>867</v>
       </c>
       <c r="P265" t="s" s="2">
         <v>78</v>
@@ -34026,13 +34069,13 @@
         <v>78</v>
       </c>
       <c r="X265" t="s" s="2">
-        <v>177</v>
+        <v>78</v>
       </c>
       <c r="Y265" t="s" s="2">
-        <v>885</v>
+        <v>78</v>
       </c>
       <c r="Z265" t="s" s="2">
-        <v>886</v>
+        <v>78</v>
       </c>
       <c r="AA265" t="s" s="2">
         <v>78</v>
@@ -34050,7 +34093,7 @@
         <v>78</v>
       </c>
       <c r="AF265" t="s" s="2">
-        <v>880</v>
+        <v>862</v>
       </c>
       <c r="AG265" t="s" s="2">
         <v>79</v>
@@ -34068,10 +34111,10 @@
         <v>78</v>
       </c>
       <c r="AL265" t="s" s="2">
-        <v>887</v>
+        <v>570</v>
       </c>
       <c r="AM265" t="s" s="2">
-        <v>109</v>
+        <v>571</v>
       </c>
       <c r="AN265" t="s" s="2">
         <v>78</v>
@@ -34080,12 +34123,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="266" hidden="true">
+    <row r="266">
       <c r="A266" t="s" s="2">
-        <v>888</v>
+        <v>868</v>
       </c>
       <c r="B266" t="s" s="2">
-        <v>888</v>
+        <v>868</v>
       </c>
       <c r="C266" s="2"/>
       <c r="D266" t="s" s="2">
@@ -34093,13 +34136,13 @@
       </c>
       <c r="E266" s="2"/>
       <c r="F266" t="s" s="2">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="G266" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H266" t="s" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="I266" t="s" s="2">
         <v>78</v>
@@ -34108,18 +34151,20 @@
         <v>78</v>
       </c>
       <c r="K266" t="s" s="2">
-        <v>812</v>
+        <v>237</v>
       </c>
       <c r="L266" t="s" s="2">
-        <v>889</v>
+        <v>869</v>
       </c>
       <c r="M266" t="s" s="2">
-        <v>890</v>
+        <v>870</v>
       </c>
       <c r="N266" t="s" s="2">
-        <v>891</v>
-      </c>
-      <c r="O266" s="2"/>
+        <v>871</v>
+      </c>
+      <c r="O266" t="s" s="2">
+        <v>872</v>
+      </c>
       <c r="P266" t="s" s="2">
         <v>78</v>
       </c>
@@ -34143,13 +34188,11 @@
         <v>78</v>
       </c>
       <c r="X266" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y266" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>327</v>
+      </c>
+      <c r="Y266" s="2"/>
       <c r="Z266" t="s" s="2">
-        <v>78</v>
+        <v>873</v>
       </c>
       <c r="AA266" t="s" s="2">
         <v>78</v>
@@ -34167,16 +34210,16 @@
         <v>78</v>
       </c>
       <c r="AF266" t="s" s="2">
-        <v>888</v>
+        <v>868</v>
       </c>
       <c r="AG266" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH266" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AI266" t="s" s="2">
-        <v>892</v>
+        <v>78</v>
       </c>
       <c r="AJ266" t="s" s="2">
         <v>103</v>
@@ -34185,10 +34228,10 @@
         <v>78</v>
       </c>
       <c r="AL266" t="s" s="2">
-        <v>893</v>
+        <v>471</v>
       </c>
       <c r="AM266" t="s" s="2">
-        <v>894</v>
+        <v>472</v>
       </c>
       <c r="AN266" t="s" s="2">
         <v>78</v>
@@ -34199,10 +34242,10 @@
     </row>
     <row r="267" hidden="true">
       <c r="A267" t="s" s="2">
-        <v>895</v>
+        <v>874</v>
       </c>
       <c r="B267" t="s" s="2">
-        <v>895</v>
+        <v>874</v>
       </c>
       <c r="C267" s="2"/>
       <c r="D267" t="s" s="2">
@@ -34213,7 +34256,7 @@
         <v>79</v>
       </c>
       <c r="G267" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="H267" t="s" s="2">
         <v>78</v>
@@ -34225,19 +34268,17 @@
         <v>78</v>
       </c>
       <c r="K267" t="s" s="2">
-        <v>237</v>
+        <v>875</v>
       </c>
       <c r="L267" t="s" s="2">
-        <v>896</v>
+        <v>876</v>
       </c>
       <c r="M267" t="s" s="2">
-        <v>897</v>
-      </c>
-      <c r="N267" t="s" s="2">
-        <v>898</v>
-      </c>
+        <v>877</v>
+      </c>
+      <c r="N267" s="2"/>
       <c r="O267" t="s" s="2">
-        <v>899</v>
+        <v>550</v>
       </c>
       <c r="P267" t="s" s="2">
         <v>78</v>
@@ -34262,13 +34303,13 @@
         <v>78</v>
       </c>
       <c r="X267" t="s" s="2">
-        <v>177</v>
+        <v>78</v>
       </c>
       <c r="Y267" t="s" s="2">
-        <v>900</v>
+        <v>78</v>
       </c>
       <c r="Z267" t="s" s="2">
-        <v>901</v>
+        <v>78</v>
       </c>
       <c r="AA267" t="s" s="2">
         <v>78</v>
@@ -34286,16 +34327,16 @@
         <v>78</v>
       </c>
       <c r="AF267" t="s" s="2">
-        <v>895</v>
+        <v>874</v>
       </c>
       <c r="AG267" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH267" t="s" s="2">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="AI267" t="s" s="2">
-        <v>892</v>
+        <v>78</v>
       </c>
       <c r="AJ267" t="s" s="2">
         <v>103</v>
@@ -34304,24 +34345,24 @@
         <v>78</v>
       </c>
       <c r="AL267" t="s" s="2">
-        <v>902</v>
+        <v>552</v>
       </c>
       <c r="AM267" t="s" s="2">
-        <v>109</v>
+        <v>553</v>
       </c>
       <c r="AN267" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AO267" t="s" s="2">
-        <v>78</v>
+        <v>555</v>
       </c>
     </row>
     <row r="268" hidden="true">
       <c r="A268" t="s" s="2">
-        <v>903</v>
+        <v>878</v>
       </c>
       <c r="B268" t="s" s="2">
-        <v>903</v>
+        <v>878</v>
       </c>
       <c r="C268" s="2"/>
       <c r="D268" t="s" s="2">
@@ -34332,7 +34373,7 @@
         <v>79</v>
       </c>
       <c r="G268" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H268" t="s" s="2">
         <v>78</v>
@@ -34344,16 +34385,16 @@
         <v>78</v>
       </c>
       <c r="K268" t="s" s="2">
-        <v>81</v>
+        <v>817</v>
       </c>
       <c r="L268" t="s" s="2">
-        <v>904</v>
+        <v>879</v>
       </c>
       <c r="M268" t="s" s="2">
-        <v>905</v>
+        <v>880</v>
       </c>
       <c r="N268" t="s" s="2">
-        <v>906</v>
+        <v>881</v>
       </c>
       <c r="O268" s="2"/>
       <c r="P268" t="s" s="2">
@@ -34403,16 +34444,16 @@
         <v>78</v>
       </c>
       <c r="AF268" t="s" s="2">
-        <v>903</v>
+        <v>878</v>
       </c>
       <c r="AG268" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH268" t="s" s="2">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="AI268" t="s" s="2">
-        <v>870</v>
+        <v>78</v>
       </c>
       <c r="AJ268" t="s" s="2">
         <v>103</v>
@@ -34421,20 +34462,728 @@
         <v>78</v>
       </c>
       <c r="AL268" t="s" s="2">
-        <v>832</v>
+        <v>78</v>
       </c>
       <c r="AM268" t="s" s="2">
+        <v>882</v>
+      </c>
+      <c r="AN268" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO268" t="s" s="2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="s" s="2">
+        <v>883</v>
+      </c>
+      <c r="B269" t="s" s="2">
+        <v>883</v>
+      </c>
+      <c r="C269" s="2"/>
+      <c r="D269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E269" s="2"/>
+      <c r="F269" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="G269" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H269" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="I269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K269" t="s" s="2">
+        <v>184</v>
+      </c>
+      <c r="L269" t="s" s="2">
+        <v>884</v>
+      </c>
+      <c r="M269" t="s" s="2">
+        <v>885</v>
+      </c>
+      <c r="N269" t="s" s="2">
+        <v>886</v>
+      </c>
+      <c r="O269" s="2"/>
+      <c r="P269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q269" s="2"/>
+      <c r="R269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF269" t="s" s="2">
+        <v>883</v>
+      </c>
+      <c r="AG269" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH269" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI269" t="s" s="2">
+        <v>887</v>
+      </c>
+      <c r="AJ269" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AK269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL269" t="s" s="2">
+        <v>888</v>
+      </c>
+      <c r="AM269" t="s" s="2">
+        <v>888</v>
+      </c>
+      <c r="AN269" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO269" t="s" s="2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="270" hidden="true">
+      <c r="A270" t="s" s="2">
+        <v>889</v>
+      </c>
+      <c r="B270" t="s" s="2">
+        <v>889</v>
+      </c>
+      <c r="C270" s="2"/>
+      <c r="D270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E270" s="2"/>
+      <c r="F270" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G270" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K270" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="L270" t="s" s="2">
+        <v>890</v>
+      </c>
+      <c r="M270" t="s" s="2">
+        <v>891</v>
+      </c>
+      <c r="N270" t="s" s="2">
+        <v>892</v>
+      </c>
+      <c r="O270" t="s" s="2">
+        <v>893</v>
+      </c>
+      <c r="P270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q270" s="2"/>
+      <c r="R270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X270" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="Y270" t="s" s="2">
+        <v>894</v>
+      </c>
+      <c r="Z270" t="s" s="2">
+        <v>895</v>
+      </c>
+      <c r="AA270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF270" t="s" s="2">
+        <v>889</v>
+      </c>
+      <c r="AG270" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH270" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ270" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AK270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL270" t="s" s="2">
+        <v>896</v>
+      </c>
+      <c r="AM270" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AN270" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO270" t="s" s="2">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="271" hidden="true">
+      <c r="A271" t="s" s="2">
+        <v>897</v>
+      </c>
+      <c r="B271" t="s" s="2">
+        <v>897</v>
+      </c>
+      <c r="C271" s="2"/>
+      <c r="D271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E271" s="2"/>
+      <c r="F271" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G271" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K271" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="L271" t="s" s="2">
+        <v>898</v>
+      </c>
+      <c r="M271" t="s" s="2">
+        <v>899</v>
+      </c>
+      <c r="N271" t="s" s="2">
+        <v>900</v>
+      </c>
+      <c r="O271" t="s" s="2">
+        <v>901</v>
+      </c>
+      <c r="P271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q271" s="2"/>
+      <c r="R271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X271" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="Y271" t="s" s="2">
+        <v>902</v>
+      </c>
+      <c r="Z271" t="s" s="2">
+        <v>903</v>
+      </c>
+      <c r="AA271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF271" t="s" s="2">
+        <v>897</v>
+      </c>
+      <c r="AG271" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH271" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ271" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AK271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL271" t="s" s="2">
+        <v>904</v>
+      </c>
+      <c r="AM271" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AN271" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO271" t="s" s="2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="272" hidden="true">
+      <c r="A272" t="s" s="2">
+        <v>905</v>
+      </c>
+      <c r="B272" t="s" s="2">
+        <v>905</v>
+      </c>
+      <c r="C272" s="2"/>
+      <c r="D272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E272" s="2"/>
+      <c r="F272" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G272" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K272" t="s" s="2">
+        <v>817</v>
+      </c>
+      <c r="L272" t="s" s="2">
+        <v>906</v>
+      </c>
+      <c r="M272" t="s" s="2">
         <v>907</v>
       </c>
-      <c r="AN268" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AO268" t="s" s="2">
+      <c r="N272" t="s" s="2">
+        <v>908</v>
+      </c>
+      <c r="O272" s="2"/>
+      <c r="P272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q272" s="2"/>
+      <c r="R272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF272" t="s" s="2">
+        <v>905</v>
+      </c>
+      <c r="AG272" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH272" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI272" t="s" s="2">
+        <v>909</v>
+      </c>
+      <c r="AJ272" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AK272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL272" t="s" s="2">
+        <v>910</v>
+      </c>
+      <c r="AM272" t="s" s="2">
+        <v>911</v>
+      </c>
+      <c r="AN272" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO272" t="s" s="2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="273" hidden="true">
+      <c r="A273" t="s" s="2">
+        <v>912</v>
+      </c>
+      <c r="B273" t="s" s="2">
+        <v>912</v>
+      </c>
+      <c r="C273" s="2"/>
+      <c r="D273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E273" s="2"/>
+      <c r="F273" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G273" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="H273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K273" t="s" s="2">
+        <v>237</v>
+      </c>
+      <c r="L273" t="s" s="2">
+        <v>913</v>
+      </c>
+      <c r="M273" t="s" s="2">
+        <v>914</v>
+      </c>
+      <c r="N273" t="s" s="2">
+        <v>915</v>
+      </c>
+      <c r="O273" t="s" s="2">
+        <v>916</v>
+      </c>
+      <c r="P273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q273" s="2"/>
+      <c r="R273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X273" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="Y273" t="s" s="2">
+        <v>917</v>
+      </c>
+      <c r="Z273" t="s" s="2">
+        <v>918</v>
+      </c>
+      <c r="AA273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF273" t="s" s="2">
+        <v>912</v>
+      </c>
+      <c r="AG273" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH273" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="AI273" t="s" s="2">
+        <v>909</v>
+      </c>
+      <c r="AJ273" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AK273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL273" t="s" s="2">
+        <v>919</v>
+      </c>
+      <c r="AM273" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AN273" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO273" t="s" s="2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="274" hidden="true">
+      <c r="A274" t="s" s="2">
+        <v>920</v>
+      </c>
+      <c r="B274" t="s" s="2">
+        <v>920</v>
+      </c>
+      <c r="C274" s="2"/>
+      <c r="D274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E274" s="2"/>
+      <c r="F274" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G274" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K274" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="L274" t="s" s="2">
+        <v>921</v>
+      </c>
+      <c r="M274" t="s" s="2">
+        <v>922</v>
+      </c>
+      <c r="N274" t="s" s="2">
+        <v>923</v>
+      </c>
+      <c r="O274" s="2"/>
+      <c r="P274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q274" s="2"/>
+      <c r="R274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF274" t="s" s="2">
+        <v>920</v>
+      </c>
+      <c r="AG274" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH274" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI274" t="s" s="2">
+        <v>887</v>
+      </c>
+      <c r="AJ274" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="AK274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AL274" t="s" s="2">
+        <v>849</v>
+      </c>
+      <c r="AM274" t="s" s="2">
+        <v>924</v>
+      </c>
+      <c r="AN274" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AO274" t="s" s="2">
         <v>78</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AO268">
+  <autoFilter ref="A1:AO274">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -34444,7 +35193,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI267">
+  <conditionalFormatting sqref="A2:AI273">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>